<commit_message>
data(sinopac): sync tax/tuition offers to official H2 2026 dates
Both offers matched the official page on all terms but were dated
H1 2026 and had expired. The bank extended the same activity to
2026/7/1-12/31, so per spec v3 rule 3.4 (same terms, longer window)
reuse the slug and update dates. Patch start/end/verified dates and
the inline dates in summary/description in the xlsx source, then
re-import; front end now shows both as active.
</commit_message>
<xml_diff>
--- a/docs/data-collection/信用卡優惠資料整理模板-v2-2026-07-18.xlsx
+++ b/docs/data-collection/信用卡優惠資料整理模板-v2-2026-07-18.xlsx
@@ -953,7 +953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.8799991607666" customWidth="1" min="1" max="1"/>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>2026-01-01 至 06-30 以 Paytax 或大咖 DACARD 繳牌照稅、房屋稅、地價稅，單筆滿 NT$3,000 登錄享 6 期 0 利率</t>
+          <t>2026-07-01 至 12-31 以 Paytax 或大咖 DACARD 繳牌照稅、房屋稅、地價稅，單筆滿 NT$3,000 登錄享 6 期 0 利率</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
@@ -2827,17 +2827,17 @@
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>2026-01-01 至 06-30，持永豐信用卡透過 Paytax 繳稅服務網（網路、QR Code 或中華電信語音）或大咖 DACARD APP 繳納牌照稅、房屋稅、地價稅；正卡持卡人完成分期總約簽署並於登錄當月繳納單筆滿 NT$3,000，登錄後可享 6 期 0 利率。指定稅款同時提供免手續費；活動另有符合歷史代繳條件者的 0.2% 刷卡金方案。</t>
+          <t>2026-07-01 至 12-31，持永豐信用卡透過 Paytax 繳稅服務網（網路、QR Code 或中華電信語音）或大咖 DACARD APP 繳納牌照稅、房屋稅、地價稅；正卡持卡人完成分期總約簽署並於登錄當月繳納單筆滿 NT$3,000，登錄後可享 6 期 0 利率。指定稅款同時提供免手續費；活動另有符合歷史代繳條件者的 0.2% 刷卡金方案。</t>
         </is>
       </c>
       <c r="I12" s="18" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="J12" s="18" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="K12" s="18" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="Q12" s="18" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R12" s="18" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>2026-01-01 至 06-30 透過 i 繳費或學費通繳學費並登錄，當月每滿 NT$50,000 回饋 NT$50，最高 NT$500</t>
+          <t>2026-07-01 至 12-31 透過 i 繳費或學費通繳學費並登錄，當月每滿 NT$50,000 回饋 NT$50，最高 NT$500</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
@@ -2920,17 +2920,17 @@
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>2026-01-01 至 06-30，透過 i 繳費或聯合信用卡中心學費通平台使用永豐信用卡繳納學費，於繳費當月完成活動登錄後，正附卡合併的當月學費每滿 NT$50,000 回饋 NT$50 刷卡金，每戶每月最高 NT$500；回饋於代繳成功次次月起入帳。另可依單筆分期活動申請 0 利率分期。</t>
+          <t>2026-07-01 至 12-31，透過 i 繳費或聯合信用卡中心學費通平台使用永豐信用卡繳納學費，於繳費當月完成活動登錄後，正附卡合併的當月學費每滿 NT$50,000 回饋 NT$50 刷卡金，每戶每月最高 NT$500；回饋於代繳成功次次月起入帳。另可依單筆分期活動申請 0 利率分期。</t>
         </is>
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="J13" s="18" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="Q13" s="18" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R13" s="18" t="inlineStr">

</xml_diff>

<commit_message>
docs(T20): draft auto scenario pages, expand core scenario tags to 14
T20 攻略文章任務卡合併「自動情境頁」與人工攻略文章方向（取代 7/27 排除自動聚合頁的決定），
並將核心情境標籤由 9 項擴充到 14 項（新增電影、高鐵台鐵、eTag、停車、道路救援），
規格書升版至 v6；CUBE 卡「玩數位」補上訂閱服務標籤，搜尋頁熱門搜尋同步加上該入口。
以上皆為文件與資料修訂，T20 本身仍是待核准草稿，未觸及 schema 或正式功能實作。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data-collection/信用卡優惠資料整理模板-v2-2026-07-18.xlsx
+++ b/docs/data-collection/信用卡優惠資料整理模板-v2-2026-07-18.xlsx
@@ -725,7 +725,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
@@ -738,7 +737,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
@@ -2157,7 +2155,7 @@
       </c>
       <c r="R4" s="18" t="inlineStr">
         <is>
-          <t>點數回饋,長期權益,指定通路,行動支付,旅遊訂房,外送,超市量販</t>
+          <t>點數回饋,長期權益,指定通路,行動支付,旅遊訂房,外送,超市量販,訂閱服務</t>
         </is>
       </c>
       <c r="S4" s="18" t="n"/>

</xml_diff>